<commit_message>
Add markdown rendering to article reader
</commit_message>
<xml_diff>
--- a/pipeline/rhemata_tracker.xlsx
+++ b/pipeline/rhemata_tracker.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Magazine Issues" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extraction" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1347,4 +1348,132 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Filename</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Pages</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Pass1</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Pass2</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Pass3</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Articles</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Pass_Count</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Warn_Count</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Flag_Count</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NewWineMagazine_Issue_03-1973.pdf</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>03-1973</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1973</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>32</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>